<commit_message>
made chanegs in designa nd added preorders section
</commit_message>
<xml_diff>
--- a/data/HW_list.xlsx
+++ b/data/HW_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C289"/>
+  <dimension ref="A1:C314"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="35.6640625" customWidth="1" min="2" max="2"/>
@@ -4238,7 +4238,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>'81 Camaro</t>
+          <t>'81 Camaro Z28</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
@@ -4754,6 +4754,381 @@
       <c r="C289" t="inlineStr">
         <is>
           <t>Silver Series Mustang 60 Years</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="n">
+        <v>289</v>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Tesla Roadster</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>Mainlines</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="n">
+        <v>290</v>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Aston Martin DB10</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>Premiums Car Culture</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="n">
+        <v>291</v>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Jaguar C-X75</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>Premiums Car Culture</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="n">
+        <v>292</v>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>'52 Hudson Hornet</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>ZAMAC</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="n">
+        <v>293</v>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Nissan 370Z</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>ZAMAC</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="n">
+        <v>294</v>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>SRT Viper GTS-R</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Mainlines</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="n">
+        <v>295</v>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Nissan Skyline GT-R V-Spec II (BNR34)</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>Premiums Car Culture</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="n">
+        <v>296</v>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Lotus Sport Elise</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>Mainlines</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="n">
+        <v>297</v>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Ferrari California</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>Mainlines</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="n">
+        <v>298</v>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Audi S4 Quattro</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>Premiums Car Culture</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="n">
+        <v>299</v>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>Audi R8 LMS</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>Premiums Car Culture</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="n">
+        <v>300</v>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>Alfa Romeo 155 V6 Ti</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>Premiums Car Culture</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="n">
+        <v>301</v>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>'69 Alfa Romeo 33 Stradale</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>Premiums Car Culture</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="n">
+        <v>302</v>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Toyota Prius Custom</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>Mainlines</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="n">
+        <v>303</v>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Ferrari 599 GTB</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>Mainlines</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="n">
+        <v>304</v>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Ferrari 12Cilindri</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>Mainlines</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="n">
+        <v>305</v>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>LB-Works Lamborghini Huracan Coupe</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Mainlines</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="n">
+        <v>306</v>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>La Liebre</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>Mainlines</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="n">
+        <v>307</v>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Honda Civic Si</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>Mainlines</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="n">
+        <v>308</v>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>Nissan Silvia (S13)</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>Fast &amp; Furious Tokyo Drift</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="n">
+        <v>309</v>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>Nissan 350z Custom</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>Fast &amp; Furious Tokyo Drift</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="n">
+        <v>310</v>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>Nissan R390 GT1</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>Mainlines</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="n">
+        <v>311</v>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Minecart</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>Mainlines</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="n">
+        <v>312</v>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Lucid Air</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>Mainlines</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="n">
+        <v>313</v>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Maserati Tipo 61</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Mainlines</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
replaced render db with supabase
</commit_message>
<xml_diff>
--- a/data/HW_list.xlsx
+++ b/data/HW_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C314"/>
+  <dimension ref="A1:C316"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="35.6640625" customWidth="1" min="2" max="2"/>
@@ -5132,6 +5132,36 @@
         </is>
       </c>
     </row>
+    <row r="315">
+      <c r="A315" t="n">
+        <v>314</v>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>TEST</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>Mainlines</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="n">
+        <v>315</v>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>TEST</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>Mainlines</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>